<commit_message>
Add post-announcement addendum; update README, FINAL_REVIEW, source log and pitch deck
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10_Supporting_Research/Support_Sources.xlsx
+++ b/10_Supporting_Research/Support_Sources.xlsx
@@ -509,7 +509,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>PURPOSE: Every source cited across this project (SRC-001 through SRC-033) is logged here with its tier classification, the specific fact it supports, and where in the project it was used — so any figure in any workbook, the pitch deck, or the information memorandum can be traced back to its origin.</t>
+          <t>PURPOSE: Every source cited across this project (SRC-001 through SRC-040) is logged here with its tier classification, the specific fact it supports, and where in the project it was used — so any figure in any workbook, the pitch deck, or the information memorandum can be traced back to its origin.</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2883,6 +2883,254 @@
         </is>
       </c>
     </row>
+    <row r="40" ht="48" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>SRC-037</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel media release, 'AkzoNobel to sell Decorative Paints South East Asia business to Nippon Paint'</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>akzonobel.com/en/media/media-releases/akzonobel-to-sell-decorative-paints-south-east-asia-business-to-nippon-paint</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>EV ~USD1.35bn (EUR1.20bn); 21x FY25 EBITDA; net proceeds ~USD1bn</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Full release (WebFetch summary, read twice)</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Buyer, seven-country perimeter, retained businesses, EV, multiple, proceeds, closing timing. No revenue or EBITDA amounts stated.</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Post_Announcement_Addendum; README; Transaction_Research (update)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>SRC-038</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel N.V. Form 6-K, Exhibit 99.1 (SEC EDGAR)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>sec.gov/Archives/edgar/data/0000003124/000095010326015189/dp254601_ex9901.htm</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (regulatory filing)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>EV ~USD1.35bn (EUR1.20bn); 21x FY25 EBITDA</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Exhibit 99.1 (WebFetch summary)</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Independently confirms EV, multiple, proceeds, countries and closing timing from the company's filing; states no revenue or EBITDA amounts.</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Post_Announcement_Addendum</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>SRC-039</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>PCI Magazine, 'AkzoNobel to sell Southeast Asia decorative paints business to Nippon Paint for $1.35 billion'</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>pcimag.com/articles/115350-akzonobel-to-sell-southeast-asia-decorative-paints-business-to-nippon-paint-for-135-billion</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials)</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>FY25 revenue ~USD291m; EBITDA ~USD65m (22%); Nippon 2026E ~16x, margin ~26%; signed 3 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Full article (WebFetch summary)</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Only source found for revenue, EBITDA, margins, 2026 projection, signing date, Dulux and Malaysian plant mentions. Single source — not confirmed elsewhere (SRC-040 did not state them). FY25 EBITDA reconciles arithmetically with 21x on USD1.35bn.</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>Tier 2 — single source for financial figures</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Post_Announcement_Addendum; README; FINAL_REVIEW s.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>SRC-040</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Business Today Malaysia (5 Oct 2026) and DealStreetAsia, coverage of the AkzoNobel / Nippon Paint SEA sale</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>businesstoday.com.my/2026/10/05/akzonobel-sells-southeast-asia-paints-business-to-nippon-paint-for-us1-35-billion/ ; dealstreetasia.com/?p=497072</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (corroboration)</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>EV ~USD1.35bn; proceeds ~USD1bn; seven countries</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Full articles (WebFetch summaries)</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Corroborate price, perimeter, proceeds and closing timing. Neither states revenue, EBITDA or advisers. Context: AkzoNobel valued the global Decorative Paints business at ~EUR7.5bn in connection with Nippon Paint's earlier approaches.</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Post_Announcement_Addendum</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post-announcement v2 model and valuation (seven countries, three cases, reverse DCF, deal check)
New 11_Post_Announcement_v2/ with a financial model and a valuation workbook built on
reported FY2024-FY2025 figures; the announced EV is used as a check, not a target.
Adds SRC-041 to SRC-046 (corroborating reports, Singapore/PNG/Australia tax rates);
updates README, FINAL_REVIEW and the addendum. September files in 01-10 unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10_Supporting_Research/Support_Sources.xlsx
+++ b/10_Supporting_Research/Support_Sources.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3131,6 +3131,378 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>SRC-041</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Investing.com, 'AkzoNobel rises as Nippon Paint buys Asia-Pacific unit for $1.35 bln' (news article)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>investing.com/news/stock-market-news/nippon-paint-shares-rise-on-135-billion-deal-for-akzos-southeast-asia-paint-arm-4930991</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials, buyer multiple)</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>FY25 revenue ~USD291m, EBITDA ~USD65m (~22%); ~16x projected 2026 EBITDA - all attributed to Nippon Paint</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Full article (search-engine excerpt; primary Nippon Paint release not read)</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Second source for FY25 revenue/EBITDA and the 16x multiple</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>SRC-042</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Singapore / MT Newswires, 'Nippon Paint to Buy AkzoNobel's Southeast Asia, Australia Units for $1.35 Billion'</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>sg.finance.yahoo.com/news/nippon-paint-buy-akzonobel-apos-014603443.html</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials)</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>FY24 revenue USD299m, EBITDA USD69m (23%); FY25 USD291m, USD65m (22%) - attributed to the Nippon Paint press release</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Full article (search-engine excerpt)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Only source found for FY24 figures besides PCI; corroborates FY25</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="48" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>SRC-043</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance UK, 'Nippon Paint shares rise on $1.35 billion deal for Akzo's Southeast Asia paint arm'</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>uk.finance.yahoo.com/news/nippon-paint-shares-rise-1-033610211.html</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials, buyer multiple)</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>FY25 revenue/EBITDA as above; ~16x 2026 EBITDA - 'Nippon Paint statement'</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Full article (search-engine excerpt)</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Corroborates FY25 figures and the 16x multiple</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>SRC-044</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>IRAS (Singapore), Corporate Income Tax Rates</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>iras.gov.sg/quick-links/tax-rates/corporate-income-tax-rates</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>2026 (accessed 2026-10-09)</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>IRAS</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Statutory corporate tax rate</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Flat 17%</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Tax rates page (search excerpt)</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Singapore CIT in the v2 blended tax</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>Tier 1 - government tax authority</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>SRC-045</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>PwC Tax Summaries, Papua New Guinea - Taxes on corporate income</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>taxsummaries.pwc.com/papua-new-guinea/corporate/taxes-on-corporate-income</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>2026 (accessed 2026-10-09)</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Papua New Guinea</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Statutory corporate tax rate</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>30% resident companies (non-resident branches 48%)</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Corporate taxes on income page (search excerpt)</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>PNG CIT in the v2 blended tax; a resident subsidiary is assumed</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>Tier 2 - professional-services tax summary</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>SRC-046</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Australian Taxation Office, Company tax rates 2025-26</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>ato.gov.au/tax-rates-and-codes/company-tax-rates/tax-rates-2025-26</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>2026 (accessed 2026-10-09)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>ATO</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Statutory corporate tax rate</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>30% standard; 25% only for base-rate entities (turnover under A$50m)</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Company tax rates page (search excerpt)</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Australia CIT in the v2 blended tax</t>
+        </is>
+      </c>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>Tier 1 - government tax authority</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix v2 Cases-sheet block overlap, correct source attribution and financials wording
Cases sheet: three case blocks overlapped (26-row spacing, 28 rows needed), overwriting
labels and leaving header text in the Base/Buyer 'terminal growth needed' cells, which
Deal_Check had pasted. Re-laid out at 31-row spacing; valuation workbook rebuilt with a
scripted pasted-value check. SRC-041 to SRC-043 re-read and corrected (Yahoo SG does not
attribute the figures to a press release). FY24/FY25 financials re-worded from
single-source to reported by several outlets, attributed to Nippon Paint; the 2026
projection stays single-source. Deck slides 2, 18, 19 edited and PDF re-exported.
No result changed. QC Addendum G added.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10_Supporting_Research/Support_Sources.xlsx
+++ b/10_Supporting_Research/Support_Sources.xlsx
@@ -3055,12 +3055,12 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>Only source found for revenue, EBITDA, margins, 2026 projection, signing date, Dulux and Malaysian plant mentions. Single source — not confirmed elsewhere (SRC-040 did not state them). FY25 EBITDA reconciles arithmetically with 21x on USD1.35bn.</t>
+          <t>First source found for revenue, EBITDA, margins, the 2026 projection, signing date, Dulux and Malaysian plant mentions (SRC-040 did not state them). FY24/FY25 revenue and EBITDA were later also found in SRC-041 to SRC-043 (reported, attributed to Nippon Paint in two of them; primary release not read). The 2026 projection (revenue above ~USD 330m, ~26% margin), signing date and Dulux/plant mentions remain single-source (this article). FY25 EBITDA reconciles arithmetically with 21x on USD1.35bn.</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>Tier 2 — single source for financial figures</t>
+          <t>Tier 2 - REPORTED financials (several outlets, see SRC-041 to SRC-043); single source for the 2026 projection</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -3169,22 +3169,22 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>FY25 revenue ~USD291m, EBITDA ~USD65m (~22%); ~16x projected 2026 EBITDA - all attributed to Nippon Paint</t>
+          <t>FY25 revenue ~USD291m, EBITDA ~USD65m, EBITDA margin 'about 22%'; 'Nippon Paint put the purchase price at roughly 16 times projected 2026 EBITDA'. The article attributes these to Nippon Paint; it does not mention a press release. No 2026 revenue/margin projection in the article.</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Full article (search-engine excerpt; primary Nippon Paint release not read)</t>
+          <t>Full article re-read 2026-10-09 (WebFetch summary; primary Nippon Paint release not read)</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>Second source for FY25 revenue/EBITDA and the 16x multiple</t>
+          <t>Second outlet for FY25 revenue/EBITDA and the ~16x multiple, attributed to Nippon Paint (no press release mentioned)</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+          <t>Tier 3 - REPORTED, attributed to Nippon Paint (basis not stated)</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -3231,22 +3231,22 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>FY24 revenue USD299m, EBITDA USD69m (23%); FY25 USD291m, USD65m (22%) - attributed to the Nippon Paint press release</t>
+          <t>FY24 revenue USD299m, EBITDA USD69m (23%); FY25 USD291m, USD65m (22%). The article gives these without naming a source in the sentence; its only 'press release' reference (Nippon Paint's funding plan) sits in an earlier paragraph. Not attributed in the article to a Nippon Paint press release.</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Full article (search-engine excerpt)</t>
+          <t>Full article re-read 2026-10-09 (WebFetch, paragraph by paragraph; primary Nippon Paint release not read)</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>Only source found for FY24 figures besides PCI; corroborates FY25</t>
+          <t>Corroborates FY25 and gives FY24 figures; NOT attributed in the article to Nippon Paint or a press release</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+          <t>Tier 3 - REPORTED, unattributed in the article</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -3293,22 +3293,22 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>FY25 revenue/EBITDA as above; ~16x 2026 EBITDA - 'Nippon Paint statement'</t>
+          <t>FY25 revenue ~USD291m, EBITDA ~USD65m, margin 'about 22%'; 'Nippon Paint put the purchase price at roughly 16 times projected 2026 EBITDA'. Attributed to Nippon Paint; no press release mentioned. No FY24 figures or 2026 revenue/margin projection.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Full article (search-engine excerpt)</t>
+          <t>Full article re-read 2026-10-09 (WebFetch summary; primary Nippon Paint release not read)</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>Corroborates FY25 figures and the 16x multiple</t>
+          <t>Third outlet for FY25 figures and the ~16x multiple, attributed to Nippon Paint (no press release mentioned)</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Tier 3 - REPORTED, attributed to Nippon Paint</t>
+          <t>Tier 3 - REPORTED, attributed to Nippon Paint (basis not stated)</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add v2 buyer analysis, transaction review deck and memo, IM status-notice copy
New in 11_Post_Announcement_v2/: buyer analysis workbook (September content unchanged,
plus outcome layer and Synergy_v2 with synergies needed to justify the price), 14-slide
transaction review deck (pptx + pdf), 4-page review memo, and a copy of the September
Information Memorandum with a status notice prepended. Adds SRC-047/SRC-048 (48 sources).
Updates READMEs, addendum, FINAL_REVIEW, QC review (Addendum H). Original deck, IM and
folders 01-10 workbooks unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10_Supporting_Research/Support_Sources.xlsx
+++ b/10_Supporting_Research/Support_Sources.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3503,6 +3503,130 @@
         </is>
       </c>
     </row>
+    <row r="50" ht="48" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>SRC-047</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Pulse 2.0, 'Nippon Paint To Acquire Akzo Nobel Decorative Paints Businesses For $1.35 Billion' (5 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>pulse2.com/nippon-paint-to-acquire-akzo-nobel-decorative-paints-businesses-for-1-35-billion/</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials, signing date)</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Seven markets; combined USD 1.35bn; FY2025 revenue ~USD 291m, EBITDA ~USD 65m (~22%); FY2024 USD 299m / USD 69m (23%); agreements signed 3 Oct 2026. Does NOT contain a 2026 revenue or margin projection.</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Full article re-read 2026-10-09 (WebFetch summary; primary release not read)</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Fourth outlet for FY24/FY25 figures (reported, attributed in the article to the acquired businesses' results; no press release named in the extract read); second source for the 3 Oct signing date; confirms the 2026 projection is not carried here</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Tier 3 - REPORTED</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="48" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>SRC-048</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Briefs Finance (briefs.co), 'Nippon Paint to Acquire Akzo Nobel's Southeast Asia Decorative Business for $1.35 Billion' (4 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>briefs.co/?p=24067</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>AkzoNobel / Nippon Paint</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Multi (SEA)</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Announced transaction (financials, multiples, synergies)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>FY2025 sales USD 291m, EBITDA USD 65m, both below the prior year (described as 'Nippon's presentation'); 'Akzo values the transaction at 21x 2025 EBITDA, whereas Nippon estimates about 16x based on its 2026 EBITDA outlook'; Nippon's earlier whole-division offer implied about 11.5x 2025 EBITDA; 'expected annual savings in the high single digits as a percentage of sales' (attribution not stated); closing targeted by mid-2027. Does NOT give a 2026 revenue or margin figure.</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Full article re-read 2026-10-09 (WebFetch summary; primary release not read)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Only source found with a synergy figure (high single-digit % of sales, attribution unclear); confirms 21x vs ~16x; confirms the 2026 projection figures are not carried here</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>Tier 3 - REPORTED</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>11_Post_Announcement_v2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>